<commit_message>
Correct NTN-B caveats in equity IRR coverage
Document that the NTN-B is taken from each source file's own columns rather than an external series, and name those columns. Record two data issues found on review: the three files never agree on the 10-year NTN-B, with utilities averaging 0.33 pp above infra, so spreads are not strictly comparable across sectors; and the malls NTN-B is wrong from Apr-2022 to Apr-2023, thirteen months rather than the four previously stated, affecting the index spread for Apr-Nov 2022. Documentation only, no data values changed.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/brazil/equity_irr/equity_irr_consolidated_coverage.xlsx
+++ b/brazil/equity_irr/equity_irr_consolidated_coverage.xlsx
@@ -670,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -896,113 +896,125 @@
     <row r="24" ht="44" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>NTN-B pairing</t>
+          <t>Where the NTN-B comes from</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>On Company Summary each name is paired with the NTN-B 10y from its own source file as of its own last date, so the spread is measured on matching dates. On the index sheet the NTN-B is the infra file where available, falling back to utilities then malls.</t>
+          <t>It is not an external series — each source file carries its own NTN-B columns, and those are what is used here. Infra: columns R/S, "10-year NTN-B" / "15-year NTN-B". Utilities: columns CQ/CR, same labels. Malls: columns X/Y, "10-year NTN-B (2035) Yield" / "15-year NTN-B (2040) Yield". On Company Summary each name is paired with the NTN-B from its OWN file as of its own last date. On the index sheet the precedence is infra, then malls; utilities is never reached, because infra spans the whole period in which utilities exists.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1">
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Q2-2022 data quality</t>
+          <t>The three files disagree on the NTN-B</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>The malls file's NTN-B dips to roughly 3-4% for four months in Q2-2022, well out of line with the ~5.7% around it. It is the only NTN-B source that far back, so the index spread (column I) is unreliable for Apr-Jul 2022. The IRR series themselves are unaffected.</t>
+          <t>Across the 389 days where infra and utilities overlap they never once agree: utilities runs on average +0.33 p.p. above infra (range +0.16 to +0.65 p.p.). The malls file pins a specific bond (NTN-B 2035) while infra and utilities say only "10-year", which would explain the drift, though the files do not state their method. CONSEQUENCE: spreads on Company Summary are not strictly comparable ACROSS sectors — utilities and sanitation names are measured against a bar about 0.33 p.p. higher than infra names, so their spreads are understated by roughly that much. Comparisons within a sector are unaffected.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1">
       <c r="B26" s="4" t="inlineStr">
         <is>
+          <t>Malls NTN-B is wrong for 13 months</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>The malls file's NTN-B reads 3.3-4.8% every month from Apr-2022 through Apr-2023, against ~5.7% before and after. Where infra overlaps this is demonstrably wrong, not merely odd: Dec-2022 reads 3.76% in malls against 6.06% in infra, Jan-2023 4.08% against 6.14%. For the INDEX the damage is confined to Apr-Nov 2022 (8 months), the window where malls is the only source; from Dec-2022 the index switches to infra. Treat the index spread (column I) as unreliable there. The IRR series themselves are unaffected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="44" customHeight="1">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
           <t>Spreads are percentage points</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Spread columns are formatted as % but are the difference between two rates: "+7.34%" means 7.34 percentage points over the bond.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="44" customHeight="1">
-      <c r="B27" s="4" t="inlineStr">
+    <row r="28" ht="44" customHeight="1">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Values, not live formulas</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Every derived figure is written as a computed value rather than a spreadsheet formula, because this environment had no LibreOffice/Excel engine available to verify formulas before delivery. The raw sheets contain the complete source series, so all of it is reproducible and auditable. Ask if you want a live-formula version.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="44" customHeight="1">
-      <c r="B28" s="4" t="inlineStr">
+    <row r="29" ht="44" customHeight="1">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Not in the source data</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>The files contain no dividend / growth / re-rating decomposition and no exit-multiple sensitivity, so neither can be built from this workbook.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="3" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>SOURCES</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="B31" s="4" t="inlineStr">
+    <row r="32" ht="18" customHeight="1">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Infra Historical IRRs.xlsx</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>https://researchxp1.s3.sa-east-1.amazonaws.com/Infra+Historical+IRRs.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="B32" s="4" t="inlineStr">
+    <row r="33" ht="18" customHeight="1">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Income Properties (Weekly).xlsb</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>https://researchxp1.s3.sa-east-1.amazonaws.com/Income+Properties+-+Historical+IRR+(Weekly).xlsb</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="B33" s="4" t="inlineStr">
+    <row r="34" ht="18" customHeight="1">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>Utilities Historical IRR.xlsx</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>https://researchxp1.s3.sa-east-1.amazonaws.com/Utilities+Historical+IRR.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="B34" s="4" t="inlineStr">
+    <row r="35" ht="18" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>Colour key</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>Blue = source data as delivered. Black = figure computed by this workbook. Shaded teal = headline number.</t>
         </is>

</xml_diff>